<commit_message>
Update CDA TS to FHIR mapping for date types 5f153a44509bfa646542dfb943f261e2781e6ef6
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaTSToDateTimeConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaTSToDateTimeConceptMap.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="43">
   <si>
     <t>Property</t>
   </si>
@@ -26,7 +26,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaTSToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaTSToDateTimeConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T14:07:48+00:00</t>
+    <t>2026-07-22T14:16:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -125,16 +125,25 @@
     <t>instant</t>
   </si>
   <si>
+    <t>Primitive Type instant</t>
+  </si>
+  <si>
     <t>http://hl7.org/fhir/StructureDefinition/dateTime|4.0.1</t>
   </si>
   <si>
     <t>dateTime</t>
   </si>
   <si>
+    <t>Primitive Type dateTime</t>
+  </si>
+  <si>
     <t>http://hl7.org/fhir/StructureDefinition/date|4.0.1</t>
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>Primitive Type date</t>
   </si>
 </sst>
 </file>
@@ -441,7 +450,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -482,7 +491,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -499,10 +508,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -543,7 +552,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -560,10 +569,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>